<commit_message>
vault backup: 2026-07-07 16:18:45
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/DC子系统模块功能拆分.xlsx
+++ b/公司项目/认知作战/文档/DC子系统模块功能拆分.xlsx
@@ -812,7 +812,7 @@
       <x:scheme val="minor"/>
     </x:font>
   </x:fonts>
-  <x:fills count="36">
+  <x:fills count="37">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1021,6 +1021,11 @@
       <x:patternFill patternType="solid">
         <x:fgColor theme="9" tint="0.399975585192419"/>
         <x:bgColor indexed="64"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="00000000"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -1278,7 +1283,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="5">
+  <x:cellXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1288,6 +1293,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="36" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1767,7 +1775,7 @@
         <x:v>22</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:8" ht="50" customHeight="1">
+    <x:row r="4" spans="1:8" ht="72" customHeight="1">
       <x:c r="A4" s="4" t="s">
         <x:v>23</x:v>
       </x:c>
@@ -1839,7 +1847,7 @@
       </x:c>
       <x:c r="H6" s="4"/>
     </x:row>
-    <x:row r="7" spans="1:8" ht="50" customHeight="1">
+    <x:row r="7" spans="1:8" ht="72" customHeight="1">
       <x:c r="A7" s="4" t="s">
         <x:v>23</x:v>
       </x:c>
@@ -2323,29 +2331,29 @@
       </x:c>
       <x:c r="H26" s="4"/>
     </x:row>
-    <x:row r="27" spans="1:8" ht="60" customHeight="1">
-      <x:c r="A27" s="3" t="str">
+    <x:row r="27" spans="1:8" ht="96" customHeight="1">
+      <x:c r="A27" s="5" t="str">
         <x:v>③功能</x:v>
       </x:c>
-      <x:c r="B27" s="3" t="str">
+      <x:c r="B27" s="5" t="str">
         <x:v>F-DC-04-04</x:v>
       </x:c>
-      <x:c r="C27" s="3" t="str">
+      <x:c r="C27" s="5" t="str">
         <x:v>采集策略自优化</x:v>
       </x:c>
-      <x:c r="D27" s="3" t="str">
+      <x:c r="D27" s="5" t="str">
         <x:v>FR-DC-002</x:v>
       </x:c>
-      <x:c r="E27" s="3" t="str">
+      <x:c r="E27" s="5" t="str">
         <x:v>基于历史采集指标对采集策略进行主动调整，使采集策略随平台反爬强度变化自适应演进，而非仅被动应对单次异常。</x:v>
       </x:c>
-      <x:c r="F27" s="3" t="str">
+      <x:c r="F27" s="5" t="str">
         <x:v>采集手段优先级排序；请求频率/并发调节；代理与账号选择策略优化；基于封禁率/成功率/反爬升级信号调整；指标波动过大维持上一稳定策略并告警</x:v>
       </x:c>
-      <x:c r="G27" s="3" t="str">
+      <x:c r="G27" s="5" t="str">
         <x:v>SRS FR-DC-002</x:v>
       </x:c>
-      <x:c r="H27" s="3" t="str">
+      <x:c r="H27" s="5" t="str">
         <x:v>补缺口④：采集→智能→优化采集的学习闭环，区别于 F-DC-04-02 的被动手段切换</x:v>
       </x:c>
     </x:row>
@@ -2638,34 +2646,84 @@
       </x:c>
       <x:c r="H40" s="4"/>
     </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="4" t="str">
+    <x:row r="41" ht="96" customHeight="1">
+      <x:c r="A41" s="3" t="str">
         <x:v>②模块</x:v>
       </x:c>
-      <x:c r="B41" s="4" t="str">
+      <x:c r="B41" s="3" t="str">
         <x:v>M-DC-07</x:v>
       </x:c>
-      <x:c r="C41" s="4" t="str">
+      <x:c r="C41" s="3" t="str">
         <x:v>情报驱动采集与目标扩散</x:v>
       </x:c>
-      <x:c r="D41" s="4" t="str">
+      <x:c r="D41" s="3" t="str">
         <x:v>FR-DC-005</x:v>
       </x:c>
-      <x:c r="E41" s="4" t="str">
+      <x:c r="E41" s="3" t="str">
         <x:v>反向驱动大脑：打通「分析→采集」反向链路，使 M-DC-06 的情报产出（目标个体/关联实体/传播节点）回注任务池并按关系扩散采集，形成「发现线索→定向扩散采集→锁定目标」的情报驱动闭环，补全认知作战最关键的反向闭环。</x:v>
       </x:c>
-      <x:c r="F41" s="4" t="str">
+      <x:c r="F41" s="3" t="str">
         <x:v>见下方功能 F-DC-07-01~02</x:v>
       </x:c>
-      <x:c r="G41" s="4" t="str">
+      <x:c r="G41" s="3" t="str">
         <x:v>SRS FR-DC-005</x:v>
       </x:c>
-      <x:c r="H41" s="4" t="str">
+      <x:c r="H41" s="3" t="str">
         <x:v>补缺口①③：闭环 M-DC-06→M-DC-01；区分 OCC「扩散趋势预判」(本期暂不实现)</x:v>
       </x:c>
     </x:row>
-    <x:row r="42"/>
-    <x:row r="43"/>
+    <x:row r="42" ht="90" customHeight="1">
+      <x:c r="A42" s="4" t="str">
+        <x:v>③功能</x:v>
+      </x:c>
+      <x:c r="B42" s="4" t="str">
+        <x:v>F-DC-07-01</x:v>
+      </x:c>
+      <x:c r="C42" s="4" t="str">
+        <x:v>情报回注采集</x:v>
+      </x:c>
+      <x:c r="D42" s="4" t="str">
+        <x:v>FR-DC-005</x:v>
+      </x:c>
+      <x:c r="E42" s="4" t="str">
+        <x:v>将 M-DC-06 分析产出的高价值目标个体、关联实体、传播节点，按回注规则自动或经人工确认生成定向采集任务(account/keyword/url_list)回注任务池，携带 source_type=intel_feedback 与来源情报标识；经 F-DC-01-03 目标级去重，命中已采集目标转为 recheck 复查而非重复采集。</x:v>
+      </x:c>
+      <x:c r="F42" s="4" t="str">
+        <x:v>情报→任务自动/人工回注；source_type=intel_feedback；目标级去重后转 recheck；人工确认闸门(高扩散/批量/敏感)；全程审计；反向接口 II-16</x:v>
+      </x:c>
+      <x:c r="G42" s="4" t="str">
+        <x:v>SRS FR-DC-005；内部接口 II-16</x:v>
+      </x:c>
+      <x:c r="H42" s="4" t="str">
+        <x:v>补缺口①：闭环「分析→采集」反向链路，把单向管道升级为情报驱动闭环</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="140" customHeight="1">
+      <x:c r="A43" s="4" t="str">
+        <x:v>③功能</x:v>
+      </x:c>
+      <x:c r="B43" s="4" t="str">
+        <x:v>F-DC-07-02</x:v>
+      </x:c>
+      <x:c r="C43" s="4" t="str">
+        <x:v>目标扩散采集</x:v>
+      </x:c>
+      <x:c r="D43" s="4" t="str">
+        <x:v>FR-DC-005</x:v>
+      </x:c>
+      <x:c r="E43" s="4" t="str">
+        <x:v>以已采集目标为起点，按指定关系类型(关注/粉丝/互动/转发链/评论链)与扩散层数图扩展式采集，每层发现的新节点经去重后生成新采集任务，形成广度优先的目标网络扩展；新目标经 ETL+分析后可再次触发回注进一步扩散，直至层数/去重命中率/人工停止，形成可控迭代扩散；受 F-DC-01-05 配额限流约束。</x:v>
+      </x:c>
+      <x:c r="F43" s="4" t="str">
+        <x:v>按关系类型+层数 BFS 扩散；新节点去重生成任务；层数/单层节点数/总数上限；迭代扩散回流；超限停止告警；区别于 OCC「扩散趋势预判」(传播预测,本期不做)</x:v>
+      </x:c>
+      <x:c r="G43" s="4" t="str">
+        <x:v>SRS FR-DC-005</x:v>
+      </x:c>
+      <x:c r="H43" s="4" t="str">
+        <x:v>补缺口③：DC 侧图扩展采集，补全「发现→扩散采集→锁定」链条；与附录 6.4 OCC 扩散趋势预判(本期暂不实现)职责区分</x:v>
+      </x:c>
+    </x:row>
     <x:row r="44"/>
   </x:sheetData>
   <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>